<commit_message>
Update project documentation and add functional test suite for demo evaluations
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/attached_assets/DEMO-PRUEBA_informe_lecciones_aprendidas_2026_T4_prueba_funcional.xlsx
+++ b/attached_assets/DEMO-PRUEBA_informe_lecciones_aprendidas_2026_T4_prueba_funcional.xlsx
@@ -445,7 +445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -518,6 +518,29 @@
         <v>Retroalimentación de prueba: la verificación previa ayuda a evitar caídas. PRUEBA FUNCIONAL PESV DEMO-PRUEBA 2026-10-11 3e7aeddd</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>26/10/2026</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>PRUEBA FUNCIONAL PESV DEMO-PRUEBA 2026-10-26 92fce0cb · Divulgación de lección aprendida</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Lección de prueba: verificar el área de tránsito antes de iniciar la jornada. PRUEBA FUNCIONAL PESV DEMO-PRUEBA 2026-10-26 92fce0cb</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>Lección de prueba: verificar el área de tránsito antes de iniciar la jornada. PRUEBA FUNCIONAL PESV DEMO-PRUEBA 2026-10-26 92fce0cb</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>PRUEBA FUNCIONAL PESV</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>26/10/2026</v>
+      </c>
+      <c r="G7" s="2" t="str">
+        <v>Retroalimentación de prueba: la verificación previa ayuda a evitar caídas. PRUEBA FUNCIONAL PESV DEMO-PRUEBA 2026-10-26 92fce0cb</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:G1"/>
@@ -525,7 +548,7 @@
     <mergeCell ref="A3:G3"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>